<commit_message>
Add validated V0/V1 history views and read-only LFE forecast API
</commit_message>
<xml_diff>
--- a/public/data/files/latest_terrain_snapshot.xlsx
+++ b/public/data/files/latest_terrain_snapshot.xlsx
@@ -754,7 +754,7 @@
         <v>46</v>
       </c>
       <c r="B2" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C2" s="2">
         <v>46304</v>
@@ -894,7 +894,7 @@
         <v>47</v>
       </c>
       <c r="B3" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C3" s="2">
         <v>46304</v>
@@ -1034,7 +1034,7 @@
         <v>48</v>
       </c>
       <c r="B4" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C4" s="2">
         <v>46304</v>
@@ -1174,7 +1174,7 @@
         <v>49</v>
       </c>
       <c r="B5" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C5" s="2">
         <v>46304</v>
@@ -1314,7 +1314,7 @@
         <v>50</v>
       </c>
       <c r="B6" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C6" s="2">
         <v>46304</v>
@@ -1454,7 +1454,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C7" s="2">
         <v>46304</v>
@@ -1594,7 +1594,7 @@
         <v>52</v>
       </c>
       <c r="B8" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C8" s="2">
         <v>46304</v>
@@ -1734,7 +1734,7 @@
         <v>53</v>
       </c>
       <c r="B9" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C9" s="2">
         <v>46304</v>
@@ -1874,7 +1874,7 @@
         <v>54</v>
       </c>
       <c r="B10" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C10" s="2">
         <v>46304</v>
@@ -2014,7 +2014,7 @@
         <v>55</v>
       </c>
       <c r="B11" s="2">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C11" s="2">
         <v>46304</v>

</xml_diff>